<commit_message>
Shadow Operation infra + S3 property pool + D2/D4 placeholder (v0.11): shadow_metrics CLI + shadow/ read-only monitor; S3 four-category proxy pool (PARTIAL, no fake READY) in structural engine; V4.6 regime_checks/verdict; D2/D4 WIND_PLACEHOLDER constant history 2018-01..2026-03 preserving real PBOC 2026-04+; wind_mapping TSF/GOV columns; fixtures+tests updated; scratch research ignored
</commit_message>
<xml_diff>
--- a/data/fixtures/wind_macro_sample.xlsx
+++ b/data/fixtures/wind_macro_sample.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="README_SYNTHETIC" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_SYNTHETIC" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,16 @@
           <t>黄金现货:SHTAU</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>社会融资规模增量</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>社融中的政府债券融资</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -496,6 +506,12 @@
       <c r="I2" t="n">
         <v>1974.014</v>
       </c>
+      <c r="J2" t="n">
+        <v>22859.1289</v>
+      </c>
+      <c r="K2" t="n">
+        <v>7238.7887</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -525,6 +541,12 @@
       <c r="I3" t="n">
         <v>1969.8804</v>
       </c>
+      <c r="J3" t="n">
+        <v>27297.0632</v>
+      </c>
+      <c r="K3" t="n">
+        <v>6575.4589</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -554,6 +576,12 @@
       <c r="I4" t="n">
         <v>1980.6606</v>
       </c>
+      <c r="J4" t="n">
+        <v>26039.582</v>
+      </c>
+      <c r="K4" t="n">
+        <v>6185.318</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -581,6 +609,12 @@
       <c r="I5" t="n">
         <v>1955.2747</v>
       </c>
+      <c r="J5" t="n">
+        <v>28078.4095</v>
+      </c>
+      <c r="K5" t="n">
+        <v>6075.1716</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -610,6 +644,12 @@
       <c r="I6" t="n">
         <v>1962.8947</v>
       </c>
+      <c r="J6" t="n">
+        <v>28204.0612</v>
+      </c>
+      <c r="K6" t="n">
+        <v>4799.9783</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -639,6 +679,12 @@
       <c r="I7" t="n">
         <v>1946.0867</v>
       </c>
+      <c r="J7" t="n">
+        <v>27740.7983</v>
+      </c>
+      <c r="K7" t="n">
+        <v>5023.4126</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -668,6 +714,12 @@
       <c r="I8" t="n">
         <v>1951.5578</v>
       </c>
+      <c r="J8" t="n">
+        <v>29695.5237</v>
+      </c>
+      <c r="K8" t="n">
+        <v>3399.1742</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -695,6 +747,12 @@
       <c r="I9" t="n">
         <v>1960.9803</v>
       </c>
+      <c r="J9" t="n">
+        <v>31469.6772</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2639.8255</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -724,6 +782,12 @@
       <c r="I10" t="n">
         <v>1987.0714</v>
       </c>
+      <c r="J10" t="n">
+        <v>23944.4965</v>
+      </c>
+      <c r="K10" t="n">
+        <v>3485.7247</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -753,6 +817,12 @@
       <c r="I11" t="n">
         <v>2041.2597</v>
       </c>
+      <c r="J11" t="n">
+        <v>27146.0727</v>
+      </c>
+      <c r="K11" t="n">
+        <v>4219.107</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -782,6 +852,12 @@
       <c r="I12" t="n">
         <v>1972.196</v>
       </c>
+      <c r="J12" t="n">
+        <v>24910.9429</v>
+      </c>
+      <c r="K12" t="n">
+        <v>3552.1197</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -810,6 +886,12 @@
       </c>
       <c r="I13" t="n">
         <v>2051.2298</v>
+      </c>
+      <c r="J13" t="n">
+        <v>24190.9203</v>
+      </c>
+      <c r="K13" t="n">
+        <v>3960.5095</v>
       </c>
     </row>
     <row r="14">
@@ -822,6 +904,8 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -851,6 +935,12 @@
       <c r="I15" t="n">
         <v>2115.4607</v>
       </c>
+      <c r="J15" t="n">
+        <v>19689.5639</v>
+      </c>
+      <c r="K15" t="n">
+        <v>5647.037</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -880,6 +970,12 @@
       <c r="I16" t="n">
         <v>2129.9841</v>
       </c>
+      <c r="J16" t="n">
+        <v>23464.3671</v>
+      </c>
+      <c r="K16" t="n">
+        <v>5749.2495</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -909,6 +1005,12 @@
       <c r="I17" t="n">
         <v>2152.2345</v>
       </c>
+      <c r="J17" t="n">
+        <v>19927.3367</v>
+      </c>
+      <c r="K17" t="n">
+        <v>6065.7496</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -938,6 +1040,12 @@
       <c r="I18" t="n">
         <v>2123.5409</v>
       </c>
+      <c r="J18" t="n">
+        <v>22509.7473</v>
+      </c>
+      <c r="K18" t="n">
+        <v>5388.9791</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -967,6 +1075,12 @@
       <c r="I19" t="n">
         <v>2072.824</v>
       </c>
+      <c r="J19" t="n">
+        <v>23963.728</v>
+      </c>
+      <c r="K19" t="n">
+        <v>5816.3143</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -996,6 +1110,12 @@
       <c r="I20" t="n">
         <v>2028.4348</v>
       </c>
+      <c r="J20" t="n">
+        <v>21158.8291</v>
+      </c>
+      <c r="K20" t="n">
+        <v>6359.6975</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -1025,6 +1145,12 @@
       <c r="I21" t="n">
         <v>2009.32</v>
       </c>
+      <c r="J21" t="n">
+        <v>23433.5482</v>
+      </c>
+      <c r="K21" t="n">
+        <v>5822.8092</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -1054,6 +1180,12 @@
       <c r="I22" t="n">
         <v>1997.8181</v>
       </c>
+      <c r="J22" t="n">
+        <v>24167.9208</v>
+      </c>
+      <c r="K22" t="n">
+        <v>5835.8373</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -1083,6 +1215,12 @@
       <c r="I23" t="n">
         <v>2036.0507</v>
       </c>
+      <c r="J23" t="n">
+        <v>24687.0116</v>
+      </c>
+      <c r="K23" t="n">
+        <v>4475.1627</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -1112,6 +1250,12 @@
       <c r="I24" t="n">
         <v>1991.3795</v>
       </c>
+      <c r="J24" t="n">
+        <v>27209.0671</v>
+      </c>
+      <c r="K24" t="n">
+        <v>4907.7759</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -1141,6 +1285,12 @@
       <c r="I25" t="n">
         <v>1998.8757</v>
       </c>
+      <c r="J25" t="n">
+        <v>25615.9424</v>
+      </c>
+      <c r="K25" t="n">
+        <v>3561.59</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -1170,6 +1320,12 @@
       <c r="I26" t="n">
         <v>2010.5505</v>
       </c>
+      <c r="J26" t="n">
+        <v>27936.2704</v>
+      </c>
+      <c r="K26" t="n">
+        <v>3387.0738</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -1199,6 +1355,12 @@
       <c r="I27" t="n">
         <v>2082.0875</v>
       </c>
+      <c r="J27" t="n">
+        <v>26482.3335</v>
+      </c>
+      <c r="K27" t="n">
+        <v>3529.1301</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -1228,6 +1390,12 @@
       <c r="I28" t="n">
         <v>2050.1871</v>
       </c>
+      <c r="J28" t="n">
+        <v>27540.9099</v>
+      </c>
+      <c r="K28" t="n">
+        <v>3595.3576</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -1257,6 +1425,12 @@
       <c r="I29" t="n">
         <v>2037.6239</v>
       </c>
+      <c r="J29" t="n">
+        <v>29504.7418</v>
+      </c>
+      <c r="K29" t="n">
+        <v>3590.9139</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -1286,6 +1460,12 @@
       <c r="I30" t="n">
         <v>1961.5341</v>
       </c>
+      <c r="J30" t="n">
+        <v>29452.5014</v>
+      </c>
+      <c r="K30" t="n">
+        <v>4545.3427</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -1315,6 +1495,12 @@
       <c r="I31" t="n">
         <v>1903.3643</v>
       </c>
+      <c r="J31" t="n">
+        <v>28858.5334</v>
+      </c>
+      <c r="K31" t="n">
+        <v>4980.07</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -1344,6 +1530,12 @@
       <c r="I32" t="n">
         <v>1887.8781</v>
       </c>
+      <c r="J32" t="n">
+        <v>24682.0493</v>
+      </c>
+      <c r="K32" t="n">
+        <v>5717.8698</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -1373,6 +1565,12 @@
       <c r="I33" t="n">
         <v>1918.7821</v>
       </c>
+      <c r="J33" t="n">
+        <v>22588.4598</v>
+      </c>
+      <c r="K33" t="n">
+        <v>6591.3714</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -1402,6 +1600,12 @@
       <c r="I34" t="n">
         <v>1910.2681</v>
       </c>
+      <c r="J34" t="n">
+        <v>23476.384</v>
+      </c>
+      <c r="K34" t="n">
+        <v>6708.2933</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -1431,6 +1635,12 @@
       <c r="I35" t="n">
         <v>1966.336</v>
       </c>
+      <c r="J35" t="n">
+        <v>21681.7079</v>
+      </c>
+      <c r="K35" t="n">
+        <v>6010.5756</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -1460,6 +1670,12 @@
       <c r="I36" t="n">
         <v>2004.5797</v>
       </c>
+      <c r="J36" t="n">
+        <v>21831.3849</v>
+      </c>
+      <c r="K36" t="n">
+        <v>6202.1145</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -1489,6 +1705,12 @@
       <c r="I37" t="n">
         <v>1968.5944</v>
       </c>
+      <c r="J37" t="n">
+        <v>21372.0298</v>
+      </c>
+      <c r="K37" t="n">
+        <v>5596.7058</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -1517,6 +1739,12 @@
       </c>
       <c r="I38" t="n">
         <v>1933.7291</v>
+      </c>
+      <c r="J38" t="n">
+        <v>19037.5186</v>
+      </c>
+      <c r="K38" t="n">
+        <v>4664.452</v>
       </c>
     </row>
   </sheetData>

</xml_diff>